<commit_message>
feat: Update monthly offline monitoring package with approved weights, spillover, 70-100 scale, and 3 tiers
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/تهیه کارنامه نواحی.xlsx
+++ b/تهیه کارنامه نواحی.xlsx
@@ -803,7 +803,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1168,6 +1168,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2990,7 +2993,7 @@
       </c>
       <c r="T30" s="41" t="inlineStr">
         <is>
-          <t>نمره کل عملکرد</t>
+          <t>نمره کل عملکرد (۷۰-۱۰۰)</t>
         </is>
       </c>
       <c r="U30" s="41" t="inlineStr">
@@ -3000,7 +3003,7 @@
       </c>
       <c r="V30" s="41" t="inlineStr">
         <is>
-          <t>سطح ارزیابی</t>
+          <t>سطح ارزیابی (۳ سطح)</t>
         </is>
       </c>
       <c r="W30" s="41" t="inlineStr">
@@ -3087,15 +3090,15 @@
         <v/>
       </c>
       <c r="T31" s="83">
-        <f>AVERAGE(F31, I31, L31, O31, R31)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F31 + 0.3*I31) + MIN(0.5, 0.5*L31 + MAX(0, 0.1*F31 + 0.3*I31 - 0.4)) + MIN(0.1, 0.1*O31)), 1)</f>
         <v/>
       </c>
       <c r="U31" s="58">
-        <f>IF(T31&gt;0, RANK(T31, $T$31:$T$62), "-")</f>
+        <f>IF(T31&gt;70, RANK(T31, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V31" s="60">
-        <f>IF(W31="فاقد گزارش", "ثبت نشده", IF(T31&gt;=1, "عالی (۱۰۰٪+)", IF(T31&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T31&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T31&lt;=70, "ضعیف", IF(T31&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W31" s="60">
@@ -3181,15 +3184,15 @@
         <v/>
       </c>
       <c r="T32" s="86">
-        <f>AVERAGE(F32, I32, L32, O32, R32)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F32 + 0.3*I32) + MIN(0.5, 0.5*L32 + MAX(0, 0.1*F32 + 0.3*I32 - 0.4)) + MIN(0.1, 0.1*O32)), 1)</f>
         <v/>
       </c>
       <c r="U32" s="62">
-        <f>IF(T32&gt;0, RANK(T32, $T$31:$T$62), "-")</f>
+        <f>IF(T32&gt;70, RANK(T32, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V32" s="64">
-        <f>IF(W32="فاقد گزارش", "ثبت نشده", IF(T32&gt;=1, "عالی (۱۰۰٪+)", IF(T32&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T32&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T32&lt;=70, "ضعیف", IF(T32&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W32" s="64">
@@ -3275,15 +3278,15 @@
         <v/>
       </c>
       <c r="T33" s="83">
-        <f>AVERAGE(F33, I33, L33, O33, R33)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F33 + 0.3*I33) + MIN(0.5, 0.5*L33 + MAX(0, 0.1*F33 + 0.3*I33 - 0.4)) + MIN(0.1, 0.1*O33)), 1)</f>
         <v/>
       </c>
       <c r="U33" s="58">
-        <f>IF(T33&gt;0, RANK(T33, $T$31:$T$62), "-")</f>
+        <f>IF(T33&gt;70, RANK(T33, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V33" s="60">
-        <f>IF(W33="فاقد گزارش", "ثبت نشده", IF(T33&gt;=1, "عالی (۱۰۰٪+)", IF(T33&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T33&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T33&lt;=70, "ضعیف", IF(T33&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W33" s="60">
@@ -3369,15 +3372,15 @@
         <v/>
       </c>
       <c r="T34" s="86">
-        <f>AVERAGE(F34, I34, L34, O34, R34)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F34 + 0.3*I34) + MIN(0.5, 0.5*L34 + MAX(0, 0.1*F34 + 0.3*I34 - 0.4)) + MIN(0.1, 0.1*O34)), 1)</f>
         <v/>
       </c>
       <c r="U34" s="62">
-        <f>IF(T34&gt;0, RANK(T34, $T$31:$T$62), "-")</f>
+        <f>IF(T34&gt;70, RANK(T34, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V34" s="64">
-        <f>IF(W34="فاقد گزارش", "ثبت نشده", IF(T34&gt;=1, "عالی (۱۰۰٪+)", IF(T34&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T34&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T34&lt;=70, "ضعیف", IF(T34&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W34" s="64">
@@ -3463,15 +3466,15 @@
         <v/>
       </c>
       <c r="T35" s="83">
-        <f>AVERAGE(F35, I35, L35, O35, R35)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F35 + 0.3*I35) + MIN(0.5, 0.5*L35 + MAX(0, 0.1*F35 + 0.3*I35 - 0.4)) + MIN(0.1, 0.1*O35)), 1)</f>
         <v/>
       </c>
       <c r="U35" s="58">
-        <f>IF(T35&gt;0, RANK(T35, $T$31:$T$62), "-")</f>
+        <f>IF(T35&gt;70, RANK(T35, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V35" s="60">
-        <f>IF(W35="فاقد گزارش", "ثبت نشده", IF(T35&gt;=1, "عالی (۱۰۰٪+)", IF(T35&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T35&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T35&lt;=70, "ضعیف", IF(T35&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W35" s="60">
@@ -3557,15 +3560,15 @@
         <v/>
       </c>
       <c r="T36" s="86">
-        <f>AVERAGE(F36, I36, L36, O36, R36)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F36 + 0.3*I36) + MIN(0.5, 0.5*L36 + MAX(0, 0.1*F36 + 0.3*I36 - 0.4)) + MIN(0.1, 0.1*O36)), 1)</f>
         <v/>
       </c>
       <c r="U36" s="62">
-        <f>IF(T36&gt;0, RANK(T36, $T$31:$T$62), "-")</f>
+        <f>IF(T36&gt;70, RANK(T36, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V36" s="64">
-        <f>IF(W36="فاقد گزارش", "ثبت نشده", IF(T36&gt;=1, "عالی (۱۰۰٪+)", IF(T36&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T36&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T36&lt;=70, "ضعیف", IF(T36&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W36" s="64">
@@ -3651,15 +3654,15 @@
         <v/>
       </c>
       <c r="T37" s="83">
-        <f>AVERAGE(F37, I37, L37, O37, R37)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F37 + 0.3*I37) + MIN(0.5, 0.5*L37 + MAX(0, 0.1*F37 + 0.3*I37 - 0.4)) + MIN(0.1, 0.1*O37)), 1)</f>
         <v/>
       </c>
       <c r="U37" s="58">
-        <f>IF(T37&gt;0, RANK(T37, $T$31:$T$62), "-")</f>
+        <f>IF(T37&gt;70, RANK(T37, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V37" s="60">
-        <f>IF(W37="فاقد گزارش", "ثبت نشده", IF(T37&gt;=1, "عالی (۱۰۰٪+)", IF(T37&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T37&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T37&lt;=70, "ضعیف", IF(T37&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W37" s="60">
@@ -3745,15 +3748,15 @@
         <v/>
       </c>
       <c r="T38" s="86">
-        <f>AVERAGE(F38, I38, L38, O38, R38)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F38 + 0.3*I38) + MIN(0.5, 0.5*L38 + MAX(0, 0.1*F38 + 0.3*I38 - 0.4)) + MIN(0.1, 0.1*O38)), 1)</f>
         <v/>
       </c>
       <c r="U38" s="62">
-        <f>IF(T38&gt;0, RANK(T38, $T$31:$T$62), "-")</f>
+        <f>IF(T38&gt;70, RANK(T38, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V38" s="64">
-        <f>IF(W38="فاقد گزارش", "ثبت نشده", IF(T38&gt;=1, "عالی (۱۰۰٪+)", IF(T38&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T38&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T38&lt;=70, "ضعیف", IF(T38&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W38" s="64">
@@ -3839,15 +3842,15 @@
         <v/>
       </c>
       <c r="T39" s="83">
-        <f>AVERAGE(F39, I39, L39, O39, R39)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F39 + 0.3*I39) + MIN(0.5, 0.5*L39 + MAX(0, 0.1*F39 + 0.3*I39 - 0.4)) + MIN(0.1, 0.1*O39)), 1)</f>
         <v/>
       </c>
       <c r="U39" s="58">
-        <f>IF(T39&gt;0, RANK(T39, $T$31:$T$62), "-")</f>
+        <f>IF(T39&gt;70, RANK(T39, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V39" s="60">
-        <f>IF(W39="فاقد گزارش", "ثبت نشده", IF(T39&gt;=1, "عالی (۱۰۰٪+)", IF(T39&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T39&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T39&lt;=70, "ضعیف", IF(T39&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W39" s="60">
@@ -3933,15 +3936,15 @@
         <v/>
       </c>
       <c r="T40" s="86">
-        <f>AVERAGE(F40, I40, L40, O40, R40)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F40 + 0.3*I40) + MIN(0.5, 0.5*L40 + MAX(0, 0.1*F40 + 0.3*I40 - 0.4)) + MIN(0.1, 0.1*O40)), 1)</f>
         <v/>
       </c>
       <c r="U40" s="62">
-        <f>IF(T40&gt;0, RANK(T40, $T$31:$T$62), "-")</f>
+        <f>IF(T40&gt;70, RANK(T40, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V40" s="64">
-        <f>IF(W40="فاقد گزارش", "ثبت نشده", IF(T40&gt;=1, "عالی (۱۰۰٪+)", IF(T40&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T40&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T40&lt;=70, "ضعیف", IF(T40&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W40" s="64">
@@ -4027,15 +4030,15 @@
         <v/>
       </c>
       <c r="T41" s="83">
-        <f>AVERAGE(F41, I41, L41, O41, R41)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F41 + 0.3*I41) + MIN(0.5, 0.5*L41 + MAX(0, 0.1*F41 + 0.3*I41 - 0.4)) + MIN(0.1, 0.1*O41)), 1)</f>
         <v/>
       </c>
       <c r="U41" s="58">
-        <f>IF(T41&gt;0, RANK(T41, $T$31:$T$62), "-")</f>
+        <f>IF(T41&gt;70, RANK(T41, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V41" s="60">
-        <f>IF(W41="فاقد گزارش", "ثبت نشده", IF(T41&gt;=1, "عالی (۱۰۰٪+)", IF(T41&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T41&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T41&lt;=70, "ضعیف", IF(T41&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W41" s="60">
@@ -4121,15 +4124,15 @@
         <v/>
       </c>
       <c r="T42" s="86">
-        <f>AVERAGE(F42, I42, L42, O42, R42)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F42 + 0.3*I42) + MIN(0.5, 0.5*L42 + MAX(0, 0.1*F42 + 0.3*I42 - 0.4)) + MIN(0.1, 0.1*O42)), 1)</f>
         <v/>
       </c>
       <c r="U42" s="62">
-        <f>IF(T42&gt;0, RANK(T42, $T$31:$T$62), "-")</f>
+        <f>IF(T42&gt;70, RANK(T42, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V42" s="64">
-        <f>IF(W42="فاقد گزارش", "ثبت نشده", IF(T42&gt;=1, "عالی (۱۰۰٪+)", IF(T42&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T42&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T42&lt;=70, "ضعیف", IF(T42&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W42" s="64">
@@ -4215,15 +4218,15 @@
         <v/>
       </c>
       <c r="T43" s="83">
-        <f>AVERAGE(F43, I43, L43, O43, R43)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F43 + 0.3*I43) + MIN(0.5, 0.5*L43 + MAX(0, 0.1*F43 + 0.3*I43 - 0.4)) + MIN(0.1, 0.1*O43)), 1)</f>
         <v/>
       </c>
       <c r="U43" s="58">
-        <f>IF(T43&gt;0, RANK(T43, $T$31:$T$62), "-")</f>
+        <f>IF(T43&gt;70, RANK(T43, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V43" s="60">
-        <f>IF(W43="فاقد گزارش", "ثبت نشده", IF(T43&gt;=1, "عالی (۱۰۰٪+)", IF(T43&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T43&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T43&lt;=70, "ضعیف", IF(T43&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W43" s="60">
@@ -4309,15 +4312,15 @@
         <v/>
       </c>
       <c r="T44" s="86">
-        <f>AVERAGE(F44, I44, L44, O44, R44)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F44 + 0.3*I44) + MIN(0.5, 0.5*L44 + MAX(0, 0.1*F44 + 0.3*I44 - 0.4)) + MIN(0.1, 0.1*O44)), 1)</f>
         <v/>
       </c>
       <c r="U44" s="62">
-        <f>IF(T44&gt;0, RANK(T44, $T$31:$T$62), "-")</f>
+        <f>IF(T44&gt;70, RANK(T44, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V44" s="64">
-        <f>IF(W44="فاقد گزارش", "ثبت نشده", IF(T44&gt;=1, "عالی (۱۰۰٪+)", IF(T44&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T44&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T44&lt;=70, "ضعیف", IF(T44&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W44" s="64">
@@ -4403,15 +4406,15 @@
         <v/>
       </c>
       <c r="T45" s="83">
-        <f>AVERAGE(F45, I45, L45, O45, R45)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F45 + 0.3*I45) + MIN(0.5, 0.5*L45 + MAX(0, 0.1*F45 + 0.3*I45 - 0.4)) + MIN(0.1, 0.1*O45)), 1)</f>
         <v/>
       </c>
       <c r="U45" s="58">
-        <f>IF(T45&gt;0, RANK(T45, $T$31:$T$62), "-")</f>
+        <f>IF(T45&gt;70, RANK(T45, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V45" s="60">
-        <f>IF(W45="فاقد گزارش", "ثبت نشده", IF(T45&gt;=1, "عالی (۱۰۰٪+)", IF(T45&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T45&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T45&lt;=70, "ضعیف", IF(T45&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W45" s="60">
@@ -4497,15 +4500,15 @@
         <v/>
       </c>
       <c r="T46" s="86">
-        <f>AVERAGE(F46, I46, L46, O46, R46)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F46 + 0.3*I46) + MIN(0.5, 0.5*L46 + MAX(0, 0.1*F46 + 0.3*I46 - 0.4)) + MIN(0.1, 0.1*O46)), 1)</f>
         <v/>
       </c>
       <c r="U46" s="62">
-        <f>IF(T46&gt;0, RANK(T46, $T$31:$T$62), "-")</f>
+        <f>IF(T46&gt;70, RANK(T46, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V46" s="64">
-        <f>IF(W46="فاقد گزارش", "ثبت نشده", IF(T46&gt;=1, "عالی (۱۰۰٪+)", IF(T46&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T46&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T46&lt;=70, "ضعیف", IF(T46&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W46" s="64">
@@ -4591,15 +4594,15 @@
         <v/>
       </c>
       <c r="T47" s="83">
-        <f>AVERAGE(F47, I47, L47, O47, R47)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F47 + 0.3*I47) + MIN(0.5, 0.5*L47 + MAX(0, 0.1*F47 + 0.3*I47 - 0.4)) + MIN(0.1, 0.1*O47)), 1)</f>
         <v/>
       </c>
       <c r="U47" s="58">
-        <f>IF(T47&gt;0, RANK(T47, $T$31:$T$62), "-")</f>
+        <f>IF(T47&gt;70, RANK(T47, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V47" s="60">
-        <f>IF(W47="فاقد گزارش", "ثبت نشده", IF(T47&gt;=1, "عالی (۱۰۰٪+)", IF(T47&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T47&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T47&lt;=70, "ضعیف", IF(T47&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W47" s="60">
@@ -4685,15 +4688,15 @@
         <v/>
       </c>
       <c r="T48" s="86">
-        <f>AVERAGE(F48, I48, L48, O48, R48)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F48 + 0.3*I48) + MIN(0.5, 0.5*L48 + MAX(0, 0.1*F48 + 0.3*I48 - 0.4)) + MIN(0.1, 0.1*O48)), 1)</f>
         <v/>
       </c>
       <c r="U48" s="62">
-        <f>IF(T48&gt;0, RANK(T48, $T$31:$T$62), "-")</f>
+        <f>IF(T48&gt;70, RANK(T48, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V48" s="64">
-        <f>IF(W48="فاقد گزارش", "ثبت نشده", IF(T48&gt;=1, "عالی (۱۰۰٪+)", IF(T48&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T48&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T48&lt;=70, "ضعیف", IF(T48&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W48" s="64">
@@ -4779,15 +4782,15 @@
         <v/>
       </c>
       <c r="T49" s="83">
-        <f>AVERAGE(F49, I49, L49, O49, R49)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F49 + 0.3*I49) + MIN(0.5, 0.5*L49 + MAX(0, 0.1*F49 + 0.3*I49 - 0.4)) + MIN(0.1, 0.1*O49)), 1)</f>
         <v/>
       </c>
       <c r="U49" s="58">
-        <f>IF(T49&gt;0, RANK(T49, $T$31:$T$62), "-")</f>
+        <f>IF(T49&gt;70, RANK(T49, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V49" s="60">
-        <f>IF(W49="فاقد گزارش", "ثبت نشده", IF(T49&gt;=1, "عالی (۱۰۰٪+)", IF(T49&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T49&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T49&lt;=70, "ضعیف", IF(T49&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W49" s="60">
@@ -4873,15 +4876,15 @@
         <v/>
       </c>
       <c r="T50" s="86">
-        <f>AVERAGE(F50, I50, L50, O50, R50)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F50 + 0.3*I50) + MIN(0.5, 0.5*L50 + MAX(0, 0.1*F50 + 0.3*I50 - 0.4)) + MIN(0.1, 0.1*O50)), 1)</f>
         <v/>
       </c>
       <c r="U50" s="62">
-        <f>IF(T50&gt;0, RANK(T50, $T$31:$T$62), "-")</f>
+        <f>IF(T50&gt;70, RANK(T50, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V50" s="64">
-        <f>IF(W50="فاقد گزارش", "ثبت نشده", IF(T50&gt;=1, "عالی (۱۰۰٪+)", IF(T50&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T50&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T50&lt;=70, "ضعیف", IF(T50&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W50" s="64">
@@ -4967,15 +4970,15 @@
         <v/>
       </c>
       <c r="T51" s="83">
-        <f>AVERAGE(F51, I51, L51, O51, R51)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F51 + 0.3*I51) + MIN(0.5, 0.5*L51 + MAX(0, 0.1*F51 + 0.3*I51 - 0.4)) + MIN(0.1, 0.1*O51)), 1)</f>
         <v/>
       </c>
       <c r="U51" s="58">
-        <f>IF(T51&gt;0, RANK(T51, $T$31:$T$62), "-")</f>
+        <f>IF(T51&gt;70, RANK(T51, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V51" s="60">
-        <f>IF(W51="فاقد گزارش", "ثبت نشده", IF(T51&gt;=1, "عالی (۱۰۰٪+)", IF(T51&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T51&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T51&lt;=70, "ضعیف", IF(T51&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W51" s="60">
@@ -5061,15 +5064,15 @@
         <v/>
       </c>
       <c r="T52" s="86">
-        <f>AVERAGE(F52, I52, L52, O52, R52)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F52 + 0.3*I52) + MIN(0.5, 0.5*L52 + MAX(0, 0.1*F52 + 0.3*I52 - 0.4)) + MIN(0.1, 0.1*O52)), 1)</f>
         <v/>
       </c>
       <c r="U52" s="62">
-        <f>IF(T52&gt;0, RANK(T52, $T$31:$T$62), "-")</f>
+        <f>IF(T52&gt;70, RANK(T52, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V52" s="64">
-        <f>IF(W52="فاقد گزارش", "ثبت نشده", IF(T52&gt;=1, "عالی (۱۰۰٪+)", IF(T52&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T52&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T52&lt;=70, "ضعیف", IF(T52&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W52" s="64">
@@ -5155,15 +5158,15 @@
         <v/>
       </c>
       <c r="T53" s="83">
-        <f>AVERAGE(F53, I53, L53, O53, R53)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F53 + 0.3*I53) + MIN(0.5, 0.5*L53 + MAX(0, 0.1*F53 + 0.3*I53 - 0.4)) + MIN(0.1, 0.1*O53)), 1)</f>
         <v/>
       </c>
       <c r="U53" s="58">
-        <f>IF(T53&gt;0, RANK(T53, $T$31:$T$62), "-")</f>
+        <f>IF(T53&gt;70, RANK(T53, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V53" s="60">
-        <f>IF(W53="فاقد گزارش", "ثبت نشده", IF(T53&gt;=1, "عالی (۱۰۰٪+)", IF(T53&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T53&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T53&lt;=70, "ضعیف", IF(T53&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W53" s="60">
@@ -5249,15 +5252,15 @@
         <v/>
       </c>
       <c r="T54" s="86">
-        <f>AVERAGE(F54, I54, L54, O54, R54)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F54 + 0.3*I54) + MIN(0.5, 0.5*L54 + MAX(0, 0.1*F54 + 0.3*I54 - 0.4)) + MIN(0.1, 0.1*O54)), 1)</f>
         <v/>
       </c>
       <c r="U54" s="62">
-        <f>IF(T54&gt;0, RANK(T54, $T$31:$T$62), "-")</f>
+        <f>IF(T54&gt;70, RANK(T54, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V54" s="64">
-        <f>IF(W54="فاقد گزارش", "ثبت نشده", IF(T54&gt;=1, "عالی (۱۰۰٪+)", IF(T54&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T54&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T54&lt;=70, "ضعیف", IF(T54&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W54" s="64">
@@ -5343,15 +5346,15 @@
         <v/>
       </c>
       <c r="T55" s="83">
-        <f>AVERAGE(F55, I55, L55, O55, R55)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F55 + 0.3*I55) + MIN(0.5, 0.5*L55 + MAX(0, 0.1*F55 + 0.3*I55 - 0.4)) + MIN(0.1, 0.1*O55)), 1)</f>
         <v/>
       </c>
       <c r="U55" s="58">
-        <f>IF(T55&gt;0, RANK(T55, $T$31:$T$62), "-")</f>
+        <f>IF(T55&gt;70, RANK(T55, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V55" s="60">
-        <f>IF(W55="فاقد گزارش", "ثبت نشده", IF(T55&gt;=1, "عالی (۱۰۰٪+)", IF(T55&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T55&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T55&lt;=70, "ضعیف", IF(T55&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W55" s="60">
@@ -5437,15 +5440,15 @@
         <v/>
       </c>
       <c r="T56" s="86">
-        <f>AVERAGE(F56, I56, L56, O56, R56)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F56 + 0.3*I56) + MIN(0.5, 0.5*L56 + MAX(0, 0.1*F56 + 0.3*I56 - 0.4)) + MIN(0.1, 0.1*O56)), 1)</f>
         <v/>
       </c>
       <c r="U56" s="62">
-        <f>IF(T56&gt;0, RANK(T56, $T$31:$T$62), "-")</f>
+        <f>IF(T56&gt;70, RANK(T56, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V56" s="64">
-        <f>IF(W56="فاقد گزارش", "ثبت نشده", IF(T56&gt;=1, "عالی (۱۰۰٪+)", IF(T56&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T56&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T56&lt;=70, "ضعیف", IF(T56&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W56" s="64">
@@ -5531,15 +5534,15 @@
         <v/>
       </c>
       <c r="T57" s="83">
-        <f>AVERAGE(F57, I57, L57, O57, R57)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F57 + 0.3*I57) + MIN(0.5, 0.5*L57 + MAX(0, 0.1*F57 + 0.3*I57 - 0.4)) + MIN(0.1, 0.1*O57)), 1)</f>
         <v/>
       </c>
       <c r="U57" s="58">
-        <f>IF(T57&gt;0, RANK(T57, $T$31:$T$62), "-")</f>
+        <f>IF(T57&gt;70, RANK(T57, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V57" s="60">
-        <f>IF(W57="فاقد گزارش", "ثبت نشده", IF(T57&gt;=1, "عالی (۱۰۰٪+)", IF(T57&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T57&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T57&lt;=70, "ضعیف", IF(T57&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W57" s="60">
@@ -5625,15 +5628,15 @@
         <v/>
       </c>
       <c r="T58" s="86">
-        <f>AVERAGE(F58, I58, L58, O58, R58)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F58 + 0.3*I58) + MIN(0.5, 0.5*L58 + MAX(0, 0.1*F58 + 0.3*I58 - 0.4)) + MIN(0.1, 0.1*O58)), 1)</f>
         <v/>
       </c>
       <c r="U58" s="62">
-        <f>IF(T58&gt;0, RANK(T58, $T$31:$T$62), "-")</f>
+        <f>IF(T58&gt;70, RANK(T58, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V58" s="64">
-        <f>IF(W58="فاقد گزارش", "ثبت نشده", IF(T58&gt;=1, "عالی (۱۰۰٪+)", IF(T58&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T58&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T58&lt;=70, "ضعیف", IF(T58&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W58" s="64">
@@ -5719,15 +5722,15 @@
         <v/>
       </c>
       <c r="T59" s="83">
-        <f>AVERAGE(F59, I59, L59, O59, R59)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F59 + 0.3*I59) + MIN(0.5, 0.5*L59 + MAX(0, 0.1*F59 + 0.3*I59 - 0.4)) + MIN(0.1, 0.1*O59)), 1)</f>
         <v/>
       </c>
       <c r="U59" s="58">
-        <f>IF(T59&gt;0, RANK(T59, $T$31:$T$62), "-")</f>
+        <f>IF(T59&gt;70, RANK(T59, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V59" s="60">
-        <f>IF(W59="فاقد گزارش", "ثبت نشده", IF(T59&gt;=1, "عالی (۱۰۰٪+)", IF(T59&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T59&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T59&lt;=70, "ضعیف", IF(T59&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W59" s="60">
@@ -5813,15 +5816,15 @@
         <v/>
       </c>
       <c r="T60" s="86">
-        <f>AVERAGE(F60, I60, L60, O60, R60)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F60 + 0.3*I60) + MIN(0.5, 0.5*L60 + MAX(0, 0.1*F60 + 0.3*I60 - 0.4)) + MIN(0.1, 0.1*O60)), 1)</f>
         <v/>
       </c>
       <c r="U60" s="62">
-        <f>IF(T60&gt;0, RANK(T60, $T$31:$T$62), "-")</f>
+        <f>IF(T60&gt;70, RANK(T60, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V60" s="64">
-        <f>IF(W60="فاقد گزارش", "ثبت نشده", IF(T60&gt;=1, "عالی (۱۰۰٪+)", IF(T60&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T60&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T60&lt;=70, "ضعیف", IF(T60&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W60" s="64">
@@ -5907,15 +5910,15 @@
         <v/>
       </c>
       <c r="T61" s="83">
-        <f>AVERAGE(F61, I61, L61, O61, R61)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F61 + 0.3*I61) + MIN(0.5, 0.5*L61 + MAX(0, 0.1*F61 + 0.3*I61 - 0.4)) + MIN(0.1, 0.1*O61)), 1)</f>
         <v/>
       </c>
       <c r="U61" s="58">
-        <f>IF(T61&gt;0, RANK(T61, $T$31:$T$62), "-")</f>
+        <f>IF(T61&gt;70, RANK(T61, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V61" s="60">
-        <f>IF(W61="فاقد گزارش", "ثبت نشده", IF(T61&gt;=1, "عالی (۱۰۰٪+)", IF(T61&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T61&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T61&lt;=70, "ضعیف", IF(T61&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W61" s="60">
@@ -6001,15 +6004,15 @@
         <v/>
       </c>
       <c r="T62" s="86">
-        <f>AVERAGE(F62, I62, L62, O62, R62)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*F62 + 0.3*I62) + MIN(0.5, 0.5*L62 + MAX(0, 0.1*F62 + 0.3*I62 - 0.4)) + MIN(0.1, 0.1*O62)), 1)</f>
         <v/>
       </c>
       <c r="U62" s="62">
-        <f>IF(T62&gt;0, RANK(T62, $T$31:$T$62), "-")</f>
+        <f>IF(T62&gt;70, RANK(T62, $T$31:$T$62), "-")</f>
         <v/>
       </c>
       <c r="V62" s="64">
-        <f>IF(W62="فاقد گزارش", "ثبت نشده", IF(T62&gt;=1, "عالی (۱۰۰٪+)", IF(T62&gt;=0.75, "خوب (۷۵-۹۹٪)", IF(T62&gt;=0.5, "متوسط (۵۰-۷۴٪)", "ضعیف (زیر ۵۰٪)"))))</f>
+        <f>IF(T62&lt;=70, "ضعیف", IF(T62&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
       <c r="W62" s="64">
@@ -6616,7 +6619,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="B1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.13" customWidth="1" style="12" min="2" max="5"/>
@@ -6654,7 +6657,7 @@
       </c>
       <c r="C3" s="135" t="inlineStr">
         <is>
-          <t>مرداد</t>
+          <t>شهریور</t>
         </is>
       </c>
       <c r="D3" s="134" t="inlineStr">
@@ -6794,11 +6797,11 @@
     <row r="11">
       <c r="B11" s="110" t="inlineStr">
         <is>
-          <t>نمره کل عملکرد:</t>
+          <t>نمره کل عملکرد (۷۰ تا ۱۰۰):</t>
         </is>
       </c>
       <c r="C11" s="111">
-        <f>AVERAGE(E5:E9)</f>
+        <f>ROUND(70 + 30 * (MIN(0.4, 0.1*E5 + 0.3*E6) + MIN(0.5, 0.5*E7 + MAX(0, 0.1*E5 + 0.3*E6 - 0.4)) + MIN(0.1, 0.1*E8)), 1)</f>
         <v/>
       </c>
       <c r="D11" s="6" t="n"/>
@@ -6820,33 +6823,44 @@
     <row r="13" ht="22" customHeight="1" s="12">
       <c r="B13" s="112" t="inlineStr">
         <is>
-          <t>سطح ارزیابی عملکرد:</t>
+          <t>سطح ارزیابی (۳ سطح):</t>
         </is>
       </c>
       <c r="C13" s="113">
-        <f>IFERROR(VLOOKUP($C$2, 'داشبورد مانیتورینگ نواحی'!$B$31:$V$62, 21, FALSE), "-")</f>
+        <f>IF(C11&lt;=70, "ضعیف", IF(C11&gt;=90, "عالی", "متوسط"))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" s="12">
       <c r="B14" s="112" t="inlineStr">
         <is>
-          <t>تعداد حوزه مقاومت:</t>
-        </is>
-      </c>
-      <c r="C14" s="114">
-        <f>IFERROR(VLOOKUP($C$2, 'پایگاه داده حد انتظار'!$A$2:$B$33, 2, FALSE), 0)</f>
+          <t>درصد تحقق وزنی اهداف:</t>
+        </is>
+      </c>
+      <c r="C14" s="140">
+        <f>(MIN(0.4, 0.1*E5 + 0.3*E6) + MIN(0.5, 0.5*E7 + MAX(0, 0.1*E5 + 0.3*E6 - 0.4)) + MIN(0.1, 0.1*E8))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" s="12">
       <c r="B15" s="112" t="inlineStr">
         <is>
+          <t>تعداد حوزه مقاومت:</t>
+        </is>
+      </c>
+      <c r="C15" s="114">
+        <f>IFERROR(VLOOKUP(, 'پایگاه داده حد انتظار'!:3, 2, FALSE), 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="0" t="inlineStr">
+        <is>
           <t>حدانتظار اعضای انجمن:</t>
         </is>
       </c>
-      <c r="C15" s="114">
-        <f>IFERROR(VLOOKUP($C$2, 'پایگاه داده حد انتظار'!$A$2:$H$33, 8, FALSE), 0)</f>
+      <c r="C16" s="0">
+        <f>IFERROR(VLOOKUP(, 'پایگاه داده حد انتظار'!:3, 8, FALSE), 0)</f>
         <v/>
       </c>
     </row>
@@ -6928,11 +6942,21 @@
           <t>آران و بیدگل</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
+      <c r="B2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -6940,11 +6964,21 @@
           <t>امام حسین(ع)</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
+      <c r="B3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -6953,7 +6987,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1064</v>
+        <v>0</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>0</v>
@@ -6965,7 +6999,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -6975,7 +7009,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>4189</v>
+        <v>0</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>0</v>
@@ -6984,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -6997,7 +7031,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>815</v>
+        <v>0</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>0</v>
@@ -7006,10 +7040,10 @@
         <v>0</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -7019,19 +7053,19 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -7044,7 +7078,7 @@
         <v>46</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>4396</v>
@@ -7062,11 +7096,21 @@
           <t>بویین و میاندشت</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
+      <c r="B9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -7074,11 +7118,21 @@
           <t>تیران و کرون</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
+      <c r="B10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -7087,7 +7141,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>0</v>
@@ -7099,7 +7153,7 @@
         <v>0</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -7108,11 +7162,21 @@
           <t>چادگان</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
+      <c r="B12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -7120,11 +7184,21 @@
           <t>خمینی شهر</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
+      <c r="B13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -7133,19 +7207,19 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>1634</v>
+        <v>0</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -7154,11 +7228,21 @@
           <t>خور و بیابانک</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -7170,13 +7254,13 @@
         <v>2299</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>1</v>
@@ -7188,11 +7272,21 @@
           <t>دهاقان</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="n"/>
+      <c r="B17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -7200,11 +7294,21 @@
           <t>سمیرم</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
+      <c r="B18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -7212,11 +7316,21 @@
           <t>شاهین شهر</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n"/>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="n"/>
+      <c r="B19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -7225,19 +7339,19 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>3366</v>
+        <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -7246,11 +7360,21 @@
           <t>فریدن</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
+      <c r="B21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -7268,10 +7392,10 @@
         <v>0</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -7281,19 +7405,19 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>1583</v>
+        <v>0</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>11348</v>
+        <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -7303,19 +7427,19 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>455</v>
+        <v>0</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -7325,19 +7449,19 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -7346,11 +7470,21 @@
           <t>گلپایگان</t>
         </is>
       </c>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
+      <c r="B26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -7359,7 +7493,7 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>0</v>
@@ -7371,7 +7505,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -7380,11 +7514,21 @@
           <t>مبارکه</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
+      <c r="B28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -7392,11 +7536,21 @@
           <t>نایین</t>
         </is>
       </c>
-      <c r="B29" s="9" t="n"/>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="n"/>
+      <c r="B29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -7404,11 +7558,21 @@
           <t>نجف آباد</t>
         </is>
       </c>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
+      <c r="B30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -7417,19 +7581,19 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>1002</v>
+        <v>0</v>
       </c>
       <c r="C31" s="9" t="n">
-        <v>187</v>
+        <v>0</v>
       </c>
       <c r="D31" s="9" t="n">
-        <v>3800</v>
+        <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F31" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -7438,11 +7602,21 @@
           <t>ورزنه</t>
         </is>
       </c>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="9" t="n"/>
-      <c r="F32" s="9" t="n"/>
+      <c r="B32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
@@ -7450,11 +7624,21 @@
           <t>هرند</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
+      <c r="B33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix NameError: unicodedata in run_aggregation and add streaming XML-repair openpyxl loader to monthly/quarterly aggregation scripts
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/تهیه کارنامه نواحی.xlsx
+++ b/تهیه کارنامه نواحی.xlsx
@@ -6657,7 +6657,7 @@
       </c>
       <c r="C3" s="135" t="inlineStr">
         <is>
-          <t>شهریور</t>
+          <t>تیر</t>
         </is>
       </c>
       <c r="D3" s="134" t="inlineStr">
@@ -7075,19 +7075,19 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>4396</v>
+        <v>0</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -7251,7 +7251,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>4552</v>
+        <v>0</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0</v>
@@ -7263,7 +7263,7 @@
         <v>0</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -7471,16 +7471,16 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>350</v>
+        <v>100</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>2170</v>
+        <v>500</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>620</v>
+        <v>400</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>1</v>

</xml_diff>